<commit_message>
Zion Cápsula (conceito, isométrica, FF&E, materiais) e marca Zion em todos os desenhos, carimbos, DXF, capas e renders
- geometry.Capsule + tools/capsule.py: prancha de conceito (planta, corte A-A, seção B-B, fachada do Visor), isométrica e lista de materiais estimados
- FF&E da Cápsula (36 itens) e item M17 cama queen; catálogo, planilha, apresentação, README e especificação atualizados para seis unidades
- svgkit.zion_mark: símbolo Z no cabeçalho e carimbo de todas as folhas SVG e detalhes, capa PA-00, títulos dos DXF, capas dos cinco documentos
- tools/brand_renders.py: renders web/deck com a marca; regen.sh atualizado (catálogo, PDF leve)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXgeeezmv3d1TAAP83TAQH
</commit_message>
<xml_diff>
--- a/projects/zion-glamping-line/ZION_MATERIAIS_FFE_Linha.xlsx
+++ b/projects/zion-glamping-line/ZION_MATERIAIS_FFE_Linha.xlsx
@@ -14,9 +14,11 @@
     <sheet name="FFE LODGE 38" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="FFE LODGE 24" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FFE LODGE 28" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Materiais Casulo" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Materiais Safari" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Materiais Lodge 38" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FFE CÁPSULA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Materiais Casulo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Materiais Safari" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Materiais Lodge 38" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Materiais Cápsula" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,12 +628,1023 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ZION CÁPSULA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cápsula monocoque transportável</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>36</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Estudo de conceito · materiais estimados por geometria</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Material / componente</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Un.</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantidade estimada</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>01 Estrutura metálica</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mastros, coroas, anéis, pilares, anel de beiral, postes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>01 Estrutura metálica</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Perfis U 150 x 60 x 3,0 galvanizados (grelha, bordas, hidromassagem)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>02 Chapas</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Chapas de base, capitéis, chapas de topo, bases articuladas, chapas de canto (D01-D14)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>03 Elementos de conexão</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Galvanização a fogo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03 Elementos de conexão</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pintura a pó (mastros, postes e anel aparentes)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>03 Elementos de conexão</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cabo de borda inox Ø12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>03 Elementos de conexão</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Estais inox Ø10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03 Elementos de conexão</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Esticadores e manilhas inox</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04 Parafusos e fixadores</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kit de parafusos, chumbadores M16/M20, pinos, contrapinos</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05 Membrana externa</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Membrana PVDF 1050 g/m² (com 15%)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05 Membrana externa</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Confecção, form-finding e padronagem dos cumes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05 Membrana externa</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Perfis de borda, clamps e trilhos de alumínio</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06 Isolamento</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lã de PET 50 mm (forro sobre o corpo)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06 Isolamento</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Manta refletiva</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06 Isolamento</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Painéis SIP 100 mm</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06 Isolamento</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Placa cimentícia + hidrófuga</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06 Isolamento</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ripado termotratado externo</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07 Membrana interna</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Forro tensionado seguindo os cumes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08 Vidros</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fachada + vidro lateral + janelas: vidro insulado low-e</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>38.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08 Vidros</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Esquadrias com ruptura térmica (fachada de correr, fixos, janelas)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>38.6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08 Vidros</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cúpula do Óculo do Zênite + esquadria</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>09 Portas</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Folhas de correr da fachada (incluídas na esquadria) + porta de correr do banho + box</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10 Deck</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Deck cumaru (terraço + passarela)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10 Deck</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Vigotas do deck</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Vigotas 50 x 150</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PIR 50 mm + manta</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Compensado naval 18 mm</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Piso de engenharia carvalho</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Zona molhada (porcelanato)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Estacas helicoidais + cabeçotes (30 + 7 de tração)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Instalação das estacas</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11 Piso</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Mobilização da cravação</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12 Banheiro</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Louças e metais (bancada dupla)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>12 Banheiro</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Banheira 1,70 m</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>12 Banheiro</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Hidromassagem Ø1,90 completa</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>12 Banheiro</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Parede da cabeceira + divisórias</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>13 Hidráulica</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Kit PEX + esgoto + ventilação</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>13 Hidráulica</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Aquecedor a gás 30 L/min</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>13 Hidráulica</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Fossa + filtro compactos</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14 Elétrica</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Quadro 16 módulos, cabos, tomadas, DR da hidromassagem</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>15 Iluminação</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Fitas LED, perfis, luminárias, balizadores do terraço</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>16 Ar-condicionado</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Dutado inverter 18k BTU instalado</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>16 Ar-condicionado</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Chaminé do Respiro motorizada + exaustor com recuperador</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17 Marcenaria</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Marcenaria sob medida (closet, Ilha do Café, bancada dupla, criados)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17 Marcenaria</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Mobiliário solto (cama, sofá, chaise, mesas)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>18 Acabamentos</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Painéis de madeira internos</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>18 Acabamentos</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Acabamentos e enxoval de abertura</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1653,13 +2666,715 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Material / componente</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Un.</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantidade estimada</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Anéis da casca: tubo retangular 60 x 40 x 3,0 mm calandrado (12 un. x 10,90 m)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>137.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Longarinas: tubo 40 x 40 x 2,0 mm curvado nas calotas (7 un.)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Chassi do piso: perfil U 150 x 50 x 3,0 mm (2 longarinas)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Travessas do piso: perfil U 100 x 50 x 2,65 mm (12 un.)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pés telescópicos: tubo Ø101,6 x 4,0 em tubo Ø114,3 x 4,5, curso 0,40 m, placa base 250 x 250 x 10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Chapas de nó, cantoneiras e olhais de içamento (4 un.)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Parafusos estruturais 8.8 galvanizados M10/M12 com porcas e arruelas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Estrutura monocoque (aço galvanizado a fogo)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Aço total estimado (anéis, longarinas, chassi, pés, chapas)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Painel de alumínio composto 4 mm (ACM) curvado, cor champanhe fosco (84,02 m² + 18 % de perdas)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>99.09999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Subestrutura do ACM: perfis ômega de alumínio 20 mm e fixadores ocultos</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>134.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Membrana de estanqueidade e barreira de vapor (manta líquida + fita butílica nas juntas)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>92.40000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Isolamento PIR 60 mm em painéis curvados entre anéis (λ 0,022)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>90.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Câmara de ar ventilada 40 mm com sarrafos de PVC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Forro e paredes: compensado naval curvado 12 mm com lâmina de carvalho, verniz fosco</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>89.59999999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Envelope (de fora para dentro)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Selante de poliuretano e fita EPDM nas juntas dos gomos</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>85.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Vidros e esquadrias (laminado curvo, alumínio anodizado bronze)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Visor: laminado curvo 8 + 8 mm low-e em 5 gomos, calandrado (11,47 m² + 10 %)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Vidros e esquadrias (laminado curvo, alumínio anodizado bronze)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Porta pivotante PV1 0,90 x 2,05 m em vidro laminado 10 + 10 com pivô e fechadura</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Vidros e esquadrias (laminado curvo, alumínio anodizado bronze)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Anel de Luz: laminado curvo 6 + 6 mm com controle solar, 3 gomos (1,74 m²)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Vidros e esquadrias (laminado curvo, alumínio anodizado bronze)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Olhos: vidro insulado circular Ø0,60 com aro de alumínio (1 transparente, 1 acidado)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Vidros e esquadrias (laminado curvo, alumínio anodizado bronze)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Vidro temperado 8 mm do box do chuveiro 0,90 x 2,00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Piso e acabamentos internos</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Painel de piso: OSB 18 mm + lã de PET 50 mm + barreira de vapor</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Piso e acabamentos internos</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Piso de carvalho de engenharia 14 mm (estar e suíte)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Piso e acabamentos internos</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Porcelanato 60 x 60 no banho, com impermeabilização</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Piso e acabamentos internos</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Parede do banho: painel SIP 90 mm com porta de correr embutida 0,80 x 2,05</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Piso e acabamentos internos</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Marcenaria fixa: closet, café/minibar, cabeceira curva, bancada do banho (ver FF&amp;E)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Deck e fundação</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Deck de cumaru 20 x 140 mm sobre vigas U 100 galvanizadas (8,32 m² + 12 %)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Deck e fundação</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Escada de três degraus em cumaru</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Deck e fundação</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Estacas helicoidais Ø76 galvanizadas com cabeçote ajustável (4 sob os pés + 4 sob o deck)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Instalações</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Elétrica: quadro 12 circuitos, 24 pontos, fita LED perimetral 2700 K, tomadas USB, iluminação do deck</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Instalações</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Hidráulica: PEX, boiler elétrico 80 L no compartimento técnico, registros, ducha, lavatório, bacia com caixa acoplada</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Instalações</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Climatização: split inverter 9.000 BTU dutado a partir do compartimento técnico, exaustor do banho</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Instalações</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ventilação: 2 grelhas de admissão nos Olhos + saída no Anel de Luz (abertura basculante motorizada)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Instalações</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Metais e louças do banho (latão escovado): ducha, misturador, cuba esculpida, bacia, acessórios</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2995,34 +4710,34 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>O01</t>
+          <t>M17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Enxoval de cama</t>
+          <t>Cama queen box + colchão</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
+          <t>Box 1,58 x 1,98 revestido em linho, colchão molas ensacadas 30 cm, pillow top (Cápsula)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>O02</t>
+          <t>O01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3032,12 +4747,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Enxoval de banho</t>
+          <t>Enxoval de cama</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
+          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3049,7 +4764,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>O03</t>
+          <t>O02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3059,12 +4774,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Amenities</t>
+          <t>Enxoval de banho</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
+          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3076,7 +4791,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>O04</t>
+          <t>O03</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3086,12 +4801,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Louças, talheres e copos</t>
+          <t>Amenities</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
+          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3103,7 +4818,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>O05</t>
+          <t>O04</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3113,12 +4828,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Manta, almofadas e decoração têxtil</t>
+          <t>Louças, talheres e copos</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
+          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3130,7 +4845,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>O06</t>
+          <t>O05</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3140,12 +4855,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Cabides, lixeiras, acessórios</t>
+          <t>Manta, almofadas e decoração têxtil</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
+          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3157,7 +4872,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>O07</t>
+          <t>O06</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3167,12 +4882,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sinalização e papelaria Zion</t>
+          <t>Cabides, lixeiras, acessórios</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Placas, diretório de serviços, QR de automação, cartões</t>
+          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3184,25 +4899,52 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>O07</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sinalização e papelaria Zion</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Placas, diretório de serviços, QR de automação, cartões</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>O08</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>Kit de segurança</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>Extintor, detector de fumaça, lanterna, kit primeiros socorros</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>cj</t>
         </is>
@@ -11540,6 +13282,1458 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Especificação</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Qtd</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Un.</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>M17</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cama queen box + colchão</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Box 1,58 x 1,98 revestido em linho, colchão molas ensacadas 30 cm, pillow top (Cápsula)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>sob o Anel de Luz, pés para o Visor</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cabeceira estofada</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Painel curvo em madeira laminada com estofado em linho, integrado à marcenaria</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>cabeceira curva na parede do banho</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Criado-mudo suspenso</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Carvalho natural, gaveta com fecho toque, iluminação embutida</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>M06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Chaise de contemplação</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Chaise 1,60 x 0,80 em madeira e corda náutica, almofada impermeável</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>chaise junto ao Visor</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>M07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Poltrona de leitura</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Poltrona giratória em couro natural e madeira</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>poltrona</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>M08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mesa de centro / lateral</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tampo em pedra (quartzito) sobre base de madeira torneada</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>mesa lateral</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>M09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ilha do café / minibar</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Marcenaria sob medida com tampo em pedra, frigobar embutido, gaveta de cápsulas</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>café / minibar 1,05 m</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Closet / armário</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Marcenaria em carvalho com portas ripadas, cabideiro, prateleiras e cofre</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>closet 1,30 x 0,40</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bancada do banho</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Tampo em pedra com cuba esculpida, gabinete ripado suspenso</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>bancada 1,20 m</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Espelho com iluminação</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Espelho redondo Ø0,90 com LED perimetral e antiembaçante</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Arandela de leitura</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Arandela articulada em latão escovado, LED 2700 K dimerizável</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Luminária de mesa</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Abajur cerâmico artesanal, 2700 K</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Tapete de lã (pequeno)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tapete de lã 1,60 x 2,30</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cortinas e blackout</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Cortina de linho + blackout motorizado, por metro linear de fachada de vidro</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Visor</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>trilho curvo no arco do Visor</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>F07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cortina da lanterna / óculo</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Tela de sombreamento motorizada circular</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Anel de Luz</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>tela motorizada curva</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Arte e objetos</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Curadoria Zion: peças de artesanato regional, cerâmica, vasos, livros</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>curadoria reduzida</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Luminárias e decoração</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Plantas e vasos</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Plantas de interior em vasos de cerâmica</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Frigobar</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Frigobar 90 L embutido, silencioso (&lt; 38 dB), classe A</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Cafeteira de cápsulas + chaleira</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cafeteira de cápsulas premium e chaleira elétrica de pescoço de ganso</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cofre eletrônico</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Cofre digital 20 L para notebook</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Closet</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Caixa de som / rádio</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sistema de som Bluetooth de mesa</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Estar</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Secador de cabelo</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Secador profissional 2000 W com suporte</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fechadura eletrônica</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Fechadura digital com cartão/senha na porta principal</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Porta PV1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Termostato e automação de cenas</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Central de automação (cenas de luz, cortinas, clima, som)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>O01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Enxoval de cama</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Suíte</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>O02</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Enxoval de banho</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>O03</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Amenities</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>O04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Louças, talheres e copos</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>O05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Manta, almofadas e decoração têxtil</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>O06</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Cabides, lixeiras, acessórios</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>O07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Sinalização e papelaria Zion</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Placas, diretório de serviços, QR de automação, cartões</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>O08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Kit de segurança</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Extintor, detector de fumaça, lanterna, kit primeiros socorros</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Deck e exterior</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Mesa e cadeiras de deck</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Mesa redonda Ø0,80 + 2 cadeiras em madeira e corda náutica</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>mesa e 2 cadeiras</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Deck e exterior</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Balizadores e lanternas de deck</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Lanternas portáteis LED recarregáveis + tochas de citronela</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Banho (acessórios)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Acessórios do banho</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Toalheiros aquecidos, ganchos, saboneteiras e porta-papel em latão escovado</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Banho (acessórios)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Balança e acessórios</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Balança digital, secador de toalhas, kit de manicure</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -12494,986 +15688,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Material / componente</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Un.</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Quantidade estimada</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>01 Estrutura metálica</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Mastros, coroas, anéis, pilares, anel de beiral, postes</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1101</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>01 Estrutura metálica</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Perfis U 150 x 60 x 3,0 galvanizados (grelha, bordas, hidromassagem)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1272</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>02 Chapas</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Chapas de base, capitéis, chapas de topo, bases articuladas, chapas de canto (D01-D14)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>03 Elementos de conexão</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Galvanização a fogo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1299</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>03 Elementos de conexão</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Pintura a pó (mastros, postes e anel aparentes)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>03 Elementos de conexão</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Cabo de borda inox Ø12</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>03 Elementos de conexão</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Estais inox Ø10</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>03 Elementos de conexão</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Esticadores e manilhas inox</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>04 Parafusos e fixadores</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Kit de parafusos, chumbadores M16/M20, pinos, contrapinos</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>kit</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>05 Membrana externa</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Membrana PVDF 1050 g/m² (com 15%)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>05 Membrana externa</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Confecção, form-finding e padronagem dos cumes</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>05 Membrana externa</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Perfis de borda, clamps e trilhos de alumínio</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>06 Isolamento</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Lã de PET 50 mm (forro sobre o corpo)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>06 Isolamento</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Manta refletiva</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>06 Isolamento</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Painéis SIP 100 mm</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>06 Isolamento</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Placa cimentícia + hidrófuga</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>06 Isolamento</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Ripado termotratado externo</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>07 Membrana interna</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Forro tensionado seguindo os cumes</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>08 Vidros</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Fachada + vidro lateral + janelas: vidro insulado low-e</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>38.6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>08 Vidros</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Esquadrias com ruptura térmica (fachada de correr, fixos, janelas)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>38.6</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>08 Vidros</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Cúpula do Óculo do Zênite + esquadria</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>09 Portas</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Folhas de correr da fachada (incluídas na esquadria) + porta de correr do banho + box</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>10 Deck</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Deck cumaru (terraço + passarela)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>10 Deck</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Vigotas do deck</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Vigotas 50 x 150</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>PIR 50 mm + manta</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Compensado naval 18 mm</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Piso de engenharia carvalho</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Zona molhada (porcelanato)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Estacas helicoidais + cabeçotes (30 + 7 de tração)</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Instalação das estacas</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>11 Piso</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Mobilização da cravação</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>vb</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>12 Banheiro</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Louças e metais (bancada dupla)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>12 Banheiro</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Banheira 1,70 m</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>12 Banheiro</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Hidromassagem Ø1,90 completa</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>12 Banheiro</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Parede da cabeceira + divisórias</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>13 Hidráulica</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Kit PEX + esgoto + ventilação</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>13 Hidráulica</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Aquecedor a gás 30 L/min</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>13 Hidráulica</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Fossa + filtro compactos</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>14 Elétrica</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Quadro 16 módulos, cabos, tomadas, DR da hidromassagem</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>15 Iluminação</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Fitas LED, perfis, luminárias, balizadores do terraço</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>16 Ar-condicionado</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Dutado inverter 18k BTU instalado</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>16 Ar-condicionado</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Chaminé do Respiro motorizada + exaustor com recuperador</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>17 Marcenaria</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Marcenaria sob medida (closet, Ilha do Café, bancada dupla, criados)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>17 Marcenaria</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Mobiliário solto (cama, sofá, chaise, mesas)</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>18 Acabamentos</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Painéis de madeira internos</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>18 Acabamentos</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Acabamentos e enxoval de abertura</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>cj</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Casulo: Bico em balanço, mini cozinha, logo oficial Zion e vídeo de órbita
- geometry.Cocoon: Bico (membrana em balanço 2,40 m sobre o deck, ponta a 4,42 m; cumeeira Ø114,3, bordas Ø60,3, costela, tirantes) em plantas, elevações, cortes, isométricas, explodido, 3D, DXF, PA, BOM e lista de peças
- Mini cozinha acoplada MA-01 (geladeira 120 L, forno 45 L, cooktop indução 2 bocas, cuba, air fryer, depurador): interiores IN-01/03/05, FF&E, circuitos C13/C14, hidráulica, textos
- Logo oficial Zion vetorizado (símbolo + logotipo horizontal) em carimbos, capas, DXF e renders
- tools/turntable.js (vídeo de órbita WebM) e 05_VIDEO/ZC-VID-001 prompts para IAs de vídeo
- regeneração completa de desenhos, renders e PDFs

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXgeeezmv3d1TAAP83TAQH
</commit_message>
<xml_diff>
--- a/projects/zion-glamping-line/ZION_MATERIAIS_FFE_Linha.xlsx
+++ b/projects/zion-glamping-line/ZION_MATERIAIS_FFE_Linha.xlsx
@@ -504,7 +504,7 @@
         <v>77.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3374,7 +3374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4008,22 +4008,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>F01</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Luminárias e decoração</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Arandela de leitura</t>
+          <t>Cooktop de indução 2 bocas</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Arandela articulada em latão escovado, LED 2700 K dimerizável</t>
+          <t>Cooktop de indução 2 zonas, 30 x 52 cm, 3,5 kW, 220 V, embutido no tampo</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -4035,22 +4035,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>E14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Luminárias e decoração</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Luminária de piso</t>
+          <t>Forno elétrico compacto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Luminária de piso em madeira e linho, 2700 K</t>
+          <t>Forno elétrico de embutir 45 L, 60 cm, 1,8 kW, porta de vidro duplo, 220 V</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4062,22 +4062,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Luminárias e decoração</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Luminária de mesa</t>
+          <t>Air fryer</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Abajur cerâmico artesanal, 2700 K</t>
+          <t>Fritadeira sem óleo 5 L, 1,5 kW, em nicho ventilado sobre o tampo</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -4089,22 +4089,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Luminárias e decoração</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tapete de lã</t>
+          <t>Geladeira sob bancada</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tapete de lã tecido à mão 2,00 x 3,00</t>
+          <t>Refrigerador 120 L sob bancada com congelador, classe A, silencioso (&lt; 40 dB), porta com painel ripado</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -4116,22 +4116,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Luminárias e decoração</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tapete de lã (pequeno)</t>
+          <t>Depurador de ar slim</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Tapete de lã 1,60 x 2,30</t>
+          <t>Depurador 60 cm com filtro de carvão ativado, 2 velocidades, LED, recirculação</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4143,7 +4143,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4153,24 +4153,24 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cortinas e blackout</t>
+          <t>Arandela de leitura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Cortina de linho + blackout motorizado, por metro linear de fachada de vidro</t>
+          <t>Arandela articulada em latão escovado, LED 2700 K dimerizável</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>F07</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4180,12 +4180,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cortina da lanterna / óculo</t>
+          <t>Luminária de piso</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Tela de sombreamento motorizada circular</t>
+          <t>Luminária de piso em madeira e linho, 2700 K</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4197,7 +4197,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>F08</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4207,24 +4207,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Arte e objetos</t>
+          <t>Luminária de mesa</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Curadoria Zion: peças de artesanato regional, cerâmica, vasos, livros</t>
+          <t>Abajur cerâmico artesanal, 2700 K</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>F09</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4234,12 +4234,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Espelho de corpo inteiro</t>
+          <t>Tapete de lã</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Espelho 0,60 x 1,80 com moldura de madeira</t>
+          <t>Tapete de lã tecido à mão 2,00 x 3,00</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4251,7 +4251,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4261,66 +4261,66 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Plantas e vasos</t>
+          <t>Tapete de lã (pequeno)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Plantas de interior em vasos de cerâmica</t>
+          <t>Tapete de lã 1,60 x 2,30</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>M01</t>
+          <t>F06</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Mobiliário</t>
+          <t>Luminárias e decoração</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cama king box + colchão</t>
+          <t>Cortinas e blackout</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Box 1,93 x 2,03 revestido em linho, colchão molas ensacadas 32 cm, pillow top</t>
+          <t>Cortina de linho + blackout motorizado, por metro linear de fachada de vidro</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>M02</t>
+          <t>F07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mobiliário</t>
+          <t>Luminárias e decoração</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Cabeceira estofada</t>
+          <t>Cortina da lanterna / óculo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Painel curvo em madeira laminada com estofado em linho, integrado à marcenaria</t>
+          <t>Tela de sombreamento motorizada circular</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -4332,49 +4332,49 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>M03</t>
+          <t>F08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mobiliário</t>
+          <t>Luminárias e decoração</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Criado-mudo suspenso</t>
+          <t>Arte e objetos</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Carvalho natural, gaveta com fecho toque, iluminação embutida</t>
+          <t>Curadoria Zion: peças de artesanato regional, cerâmica, vasos, livros</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>vb</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>M04</t>
+          <t>F09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mobiliário</t>
+          <t>Luminárias e decoração</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sofá 2,40 m</t>
+          <t>Espelho de corpo inteiro</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Estrutura em madeira, espuma D33, tecido bouclé antimancha</t>
+          <t>Espelho 0,60 x 1,80 com moldura de madeira</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4386,34 +4386,34 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>M05</t>
+          <t>F10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mobiliário</t>
+          <t>Luminárias e decoração</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sofá 2,00 m</t>
+          <t>Plantas e vasos</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Estrutura em madeira, espuma D33, tecido bouclé antimancha</t>
+          <t>Plantas de interior em vasos de cerâmica</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>vb</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>M06</t>
+          <t>M01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4423,12 +4423,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Chaise de contemplação</t>
+          <t>Cama king box + colchão</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Chaise 1,60 x 0,80 em madeira e corda náutica, almofada impermeável</t>
+          <t>Box 1,93 x 2,03 revestido em linho, colchão molas ensacadas 32 cm, pillow top</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4440,7 +4440,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>M07</t>
+          <t>M02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4450,12 +4450,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Poltrona de leitura</t>
+          <t>Cabeceira estofada</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Poltrona giratória em couro natural e madeira</t>
+          <t>Painel curvo em madeira laminada com estofado em linho, integrado à marcenaria</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4467,7 +4467,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>M08</t>
+          <t>M03</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4477,12 +4477,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mesa de centro / lateral</t>
+          <t>Criado-mudo suspenso</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Tampo em pedra (quartzito) sobre base de madeira torneada</t>
+          <t>Carvalho natural, gaveta com fecho toque, iluminação embutida</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4494,7 +4494,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>M09</t>
+          <t>M04</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4504,12 +4504,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ilha do café / minibar</t>
+          <t>Sofá 2,40 m</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Marcenaria sob medida com tampo em pedra, frigobar embutido, gaveta de cápsulas</t>
+          <t>Estrutura em madeira, espuma D33, tecido bouclé antimancha</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4521,7 +4521,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4531,12 +4531,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Closet / armário</t>
+          <t>Sofá 2,00 m</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Marcenaria em carvalho com portas ripadas, cabideiro, prateleiras e cofre</t>
+          <t>Estrutura em madeira, espuma D33, tecido bouclé antimancha</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4548,7 +4548,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M06</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4558,12 +4558,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Banco aos pés da cama</t>
+          <t>Chaise de contemplação</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Banco 1,40 m em madeira e couro</t>
+          <t>Chaise 1,60 x 0,80 em madeira e corda náutica, almofada impermeável</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4575,7 +4575,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>M12</t>
+          <t>M07</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4585,12 +4585,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bancada do banho</t>
+          <t>Poltrona de leitura</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Tampo em pedra com cuba esculpida, gabinete ripado suspenso</t>
+          <t>Poltrona giratória em couro natural e madeira</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4602,7 +4602,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4612,12 +4612,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Espelho com iluminação</t>
+          <t>Mesa de centro / lateral</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Espelho redondo Ø0,90 com LED perimetral e antiembaçante</t>
+          <t>Tampo em pedra (quartzito) sobre base de madeira torneada</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4629,7 +4629,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>M14</t>
+          <t>M09</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4639,24 +4639,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mesa de refeições / trabalho</t>
+          <t>Ilha do café / minibar</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Mesa 0,80 x 1,20 em carvalho + 2 cadeiras</t>
+          <t>Marcenaria sob medida com tampo em pedra, frigobar embutido, gaveta de cápsulas</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>M15</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -4666,12 +4666,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Totem do mastro (Safari)</t>
+          <t>Closet / armário</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Revestimento do mastro M2 em madeira com prateleiras e iluminação</t>
+          <t>Marcenaria em carvalho com portas ripadas, cabideiro, prateleiras e cofre</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4683,7 +4683,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>M16</t>
+          <t>M11</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4693,24 +4693,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ripado da cabeceira</t>
+          <t>Banco aos pés da cama</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Painel ripado termotratado com fitas LED (parede da cabeceira)</t>
+          <t>Banco 1,40 m em madeira e couro</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>M17</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4720,12 +4720,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Cama queen box + colchão</t>
+          <t>Bancada do banho</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Box 1,58 x 1,98 revestido em linho, colchão molas ensacadas 30 cm, pillow top (Cápsula)</t>
+          <t>Tampo em pedra com cuba esculpida, gabinete ripado suspenso</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4737,49 +4737,49 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>O01</t>
+          <t>M13</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Enxoval de cama</t>
+          <t>Espelho com iluminação</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
+          <t>Espelho redondo Ø0,90 com LED perimetral e antiembaçante</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>O02</t>
+          <t>M14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Enxoval de banho</t>
+          <t>Mesa de refeições / trabalho</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
+          <t>Mesa 0,80 x 1,20 em carvalho + 2 cadeiras</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4791,115 +4791,115 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>O03</t>
+          <t>M15</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Amenities</t>
+          <t>Totem do mastro (Safari)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
+          <t>Revestimento do mastro M2 em madeira com prateleiras e iluminação</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>O04</t>
+          <t>M16</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Louças, talheres e copos</t>
+          <t>Ripado da cabeceira</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
+          <t>Painel ripado termotratado com fitas LED (parede da cabeceira)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>m²</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>O05</t>
+          <t>M17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Manta, almofadas e decoração têxtil</t>
+          <t>Cama queen box + colchão</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
+          <t>Box 1,58 x 1,98 revestido em linho, colchão molas ensacadas 30 cm, pillow top (Cápsula)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>O06</t>
+          <t>M18</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Mobiliário</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Cabides, lixeiras, acessórios</t>
+          <t>Mini cozinha acoplada</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
+          <t>Marcenaria sob medida 2,00 m acoplada à concha: tampo em quartzito, cuba, módulos para geladeira, forno, gaveteiro e lixeira, prateleira com LED (Casulo)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>O07</t>
+          <t>O01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4909,12 +4909,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sinalização e papelaria Zion</t>
+          <t>Enxoval de cama</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Placas, diretório de serviços, QR de automação, cartões</t>
+          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -4926,25 +4926,214 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>O02</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Enxoval de banho</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>O03</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Amenities</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>O04</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Louças, talheres e copos</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>O05</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Manta, almofadas e decoração têxtil</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>O06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Cabides, lixeiras, acessórios</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>O07</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Sinalização e papelaria Zion</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Placas, diretório de serviços, QR de automação, cartões</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>O08</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>Kit de segurança</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>Extintor, detector de fumaça, lanterna, kit primeiros socorros</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>O09</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Enxoval e OS&amp;E</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Utensílios de cozinha</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Jogo de panelas para indução, frigideira, tábua, facas, utensílios, escorredor, potes</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>cj</t>
         </is>
@@ -4961,7 +5150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5337,7 +5526,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M09</t>
+          <t>M18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5347,12 +5536,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ilha do café / minibar</t>
+          <t>Mini cozinha acoplada</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Marcenaria sob medida com tampo em pedra, frigobar embutido, gaveta de cápsulas</t>
+          <t>Marcenaria sob medida 2,00 m acoplada à concha: tampo em quartzito, cuba, módulos para geladeira, forno, gaveteiro e lixeira, prateleira com LED (Casulo)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5362,7 +5551,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>café / minibar 1,40 m</t>
+          <t>mini cozinha 2,00 m</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -5403,7 +5592,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>armário baixo embutido 1,40 m</t>
+          <t>armário baixo embutido 1,10 m</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -5838,7 +6027,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5848,20 +6037,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Frigobar</t>
+          <t>Geladeira sob bancada</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Frigobar 90 L embutido, silencioso (&lt; 38 dB), classe A</t>
+          <t>Refrigerador 120 L sob bancada com congelador, classe A, silencioso (&lt; 40 dB), porta com painel ripado</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Estar</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>Mini cozinha</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>sob bancada</t>
+        </is>
+      </c>
       <c r="G23" t="n">
         <v>1</v>
       </c>
@@ -5875,7 +6068,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5885,26 +6078,30 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Cafeteira de cápsulas + chaleira</t>
+          <t>Cooktop de indução 2 bocas</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cafeteira de cápsulas premium e chaleira elétrica de pescoço de ganso</t>
+          <t>Cooktop de indução 2 zonas, 30 x 52 cm, 3,5 kW, 220 V, embutido no tampo</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Estar</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>Mini cozinha</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>circuito dedicado C13</t>
+        </is>
+      </c>
       <c r="G24" t="n">
         <v>1</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -5912,7 +6109,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5922,20 +6119,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cofre eletrônico</t>
+          <t>Forno elétrico compacto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Cofre digital 20 L para notebook</t>
+          <t>Forno elétrico de embutir 45 L, 60 cm, 1,8 kW, porta de vidro duplo, 220 V</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Armário</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>Mini cozinha</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>circuito dedicado C14</t>
+        </is>
+      </c>
       <c r="G25" t="n">
         <v>1</v>
       </c>
@@ -5949,7 +6150,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5959,17 +6160,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Caixa de som / rádio</t>
+          <t>Air fryer</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sistema de som Bluetooth de mesa</t>
+          <t>Fritadeira sem óleo 5 L, 1,5 kW, em nicho ventilado sobre o tampo</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Estar</t>
+          <t>Mini cozinha</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -5986,7 +6187,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5996,17 +6197,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Secador de cabelo</t>
+          <t>Depurador de ar slim</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Secador profissional 2000 W com suporte</t>
+          <t>Depurador 60 cm com filtro de carvão ativado, 2 velocidades, LED, recirculação</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Banho</t>
+          <t>Mini cozinha</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -6023,7 +6224,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6033,17 +6234,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Aquecedor / lareira ecológica</t>
+          <t>Cafeteira de cápsulas + chaleira</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Lareira a etanol de mesa ou de piso (inverno)</t>
+          <t>Cafeteira de cápsulas premium e chaleira elétrica de pescoço de ganso</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Estar</t>
+          <t>Mini cozinha</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -6052,7 +6253,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>cj</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -6060,7 +6261,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6070,17 +6271,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fechadura eletrônica</t>
+          <t>Cofre eletrônico</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Fechadura digital com cartão/senha na porta principal</t>
+          <t>Cofre digital 20 L para notebook</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Porta PV1</t>
+          <t>Armário</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -6097,7 +6298,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6107,17 +6308,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Termostato e automação de cenas</t>
+          <t>Caixa de som / rádio</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Central de automação (cenas de luz, cortinas, clima, som)</t>
+          <t>Sistema de som Bluetooth de mesa</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ático técnico</t>
+          <t>Estar</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -6134,27 +6335,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>O01</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Enxoval de cama</t>
+          <t>Secador de cabelo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
+          <t>Secador profissional 2000 W com suporte</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Suíte</t>
+          <t>Banho</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -6163,7 +6364,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -6171,27 +6372,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>O02</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Enxoval de banho</t>
+          <t>Aquecedor / lareira ecológica</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
+          <t>Lareira a etanol de mesa ou de piso (inverno)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Banho</t>
+          <t>Estar</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -6200,7 +6401,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -6208,27 +6409,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>O03</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Amenities</t>
+          <t>Fechadura eletrônica</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
+          <t>Fechadura digital com cartão/senha na porta principal</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Banho</t>
+          <t>Porta PV1</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -6237,7 +6438,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -6245,27 +6446,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>O04</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Enxoval e OS&amp;E</t>
+          <t>Equipamentos</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Louças, talheres e copos</t>
+          <t>Termostato e automação de cenas</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
+          <t>Central de automação (cenas de luz, cortinas, clima, som)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Ático técnico</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -6274,7 +6475,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>un</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -6282,7 +6483,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>O05</t>
+          <t>O01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6292,17 +6493,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Manta, almofadas e decoração têxtil</t>
+          <t>Enxoval de cama</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
+          <t>3 jogos: lençóis 400 fios algodão egípcio, edredom, duvet, protetor, 6 travesseiros</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Suíte</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -6319,7 +6520,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>O06</t>
+          <t>O02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6329,17 +6530,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Cabides, lixeiras, acessórios</t>
+          <t>Enxoval de banho</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
+          <t>3 jogos: toalhas de banho/rosto/piso 600 g/m², roupões, chinelos</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Banho</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -6356,7 +6557,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>O07</t>
+          <t>O03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6366,17 +6567,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sinalização e papelaria Zion</t>
+          <t>Amenities</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Placas, diretório de serviços, QR de automação, cartões</t>
+          <t>Dispensers de vidro (shampoo, condicionador, sabonete, hidratante) + kit de boas-vindas (estoque inicial)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Banho</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -6393,7 +6594,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>O08</t>
+          <t>O04</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6403,17 +6604,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Kit de segurança</t>
+          <t>Louças, talheres e copos</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Extintor, detector de fumaça, lanterna, kit primeiros socorros</t>
+          <t>Serviço para 4 (café da manhã e taças de vinho), bandeja, cesta</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Mini cozinha</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -6430,27 +6631,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>O09</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Deck e exterior</t>
+          <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Espreguiçadeiras</t>
+          <t>Utensílios de cozinha</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Par de espreguiçadeiras em madeira teca e corda náutica, almofadas outdoor</t>
+          <t>Jogo de panelas para indução, frigideira, tábua, facas, utensílios, escorredor, potes</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Deck</t>
+          <t>Mini cozinha</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -6459,7 +6660,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>par</t>
+          <t>cj</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -6467,27 +6668,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>O05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Deck e exterior</t>
+          <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mesa e cadeiras de deck</t>
+          <t>Manta, almofadas e decoração têxtil</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Mesa redonda Ø0,80 + 2 cadeiras em madeira e corda náutica</t>
+          <t>Manta de lã, 6 almofadas, cortina de banho em linho</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Deck</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -6504,27 +6705,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>O06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Deck e exterior</t>
+          <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Balizadores e lanternas de deck</t>
+          <t>Cabides, lixeiras, acessórios</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Lanternas portáteis LED recarregáveis + tochas de citronela</t>
+          <t>Cabides de madeira, lixeiras, cesto de roupa, kit de costura, guarda-chuva</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Deck</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -6541,27 +6742,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>O07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Deck e exterior</t>
+          <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ducha externa</t>
+          <t>Sinalização e papelaria Zion</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Ducha de deck em aço inox com base de cumaru</t>
+          <t>Placas, diretório de serviços, QR de automação, cartões</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Deck</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -6570,7 +6771,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>cj</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -6578,72 +6779,64 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>O08</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Equipamentos</t>
+          <t>Enxoval e OS&amp;E</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Hidromassagem externa</t>
+          <t>Kit de segurança</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Hot tub de 4 lugares, fibra, aquecimento a gás/elétrico, cobertura térmica</t>
+          <t>Extintor, detector de fumaça, lanterna, kit primeiros socorros</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Deck</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>opcional: hot tub Ø1,90 no deck</t>
-        </is>
-      </c>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
         <v>1</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>opcional</t>
-        </is>
-      </c>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Banho (acessórios)</t>
+          <t>Deck e exterior</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Acessórios do banho</t>
+          <t>Espreguiçadeiras</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Toalheiros aquecidos, ganchos, saboneteiras e porta-papel em latão escovado</t>
+          <t>Par de espreguiçadeiras em madeira teca e corda náutica, almofadas outdoor</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Banho</t>
+          <t>Deck</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -6652,7 +6845,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>cj</t>
+          <t>par</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -6660,34 +6853,30 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Banho (acessórios)</t>
+          <t>Deck e exterior</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Banqueta e bandeja da banheira</t>
+          <t>Mesa e cadeiras de deck</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Banqueta de teca e bandeja para banheira</t>
+          <t>Mesa redonda Ø0,80 + 2 cadeiras em madeira e corda náutica</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Banho</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>banheira 1,60</t>
-        </is>
-      </c>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
         <v>1</v>
       </c>
@@ -6701,27 +6890,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Banho (acessórios)</t>
+          <t>Deck e exterior</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Balança e acessórios</t>
+          <t>Balizadores e lanternas de deck</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Balança digital, secador de toalhas, kit de manicure</t>
+          <t>Lanternas portáteis LED recarregáveis + tochas de citronela</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Banho</t>
+          <t>Deck</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -6734,6 +6923,203 @@
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Deck e exterior</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Ducha externa</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Ducha de deck em aço inox com base de cumaru</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Hidromassagem externa</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Hot tub de 4 lugares, fibra, aquecimento a gás/elétrico, cobertura térmica</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>opcional: hot tub Ø1,90 no deck</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>opcional</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Banho (acessórios)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Acessórios do banho</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Toalheiros aquecidos, ganchos, saboneteiras e porta-papel em latão escovado</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Banho (acessórios)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Banqueta e bandeja da banheira</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Banqueta de teca e bandeja para banheira</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>banheira 1,60</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Banho (acessórios)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Balança e acessórios</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Balança digital, secador de toalhas, kit de manicure</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Banho</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14782,7 +15168,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1128</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="3">
@@ -14842,7 +15228,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1340</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="6">
@@ -14862,7 +15248,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>938</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="7">
@@ -14942,7 +15328,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11">
@@ -14962,7 +15348,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12">
@@ -15022,7 +15408,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15">
@@ -15042,7 +15428,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16">
@@ -15062,7 +15448,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17">
@@ -15082,7 +15468,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Lotes por modelo, padrões de corte das lonas, master plan e one-pager
- tools/lona.py: planificação por tiras entre costuras para Casulo, Safari, Lodge 38 e Cápsula (lona externa, forro, revestimento): pranchas LN-01/LN-1n/LN-90, DXF e XLSX por modelo
- tools/build_lotes.py: 16 documentos de lote (deck e infra, estrutura metálica, lonas/revestimentos/vidros, mobílias) x 4 modelos, ZG-MP-001 master plan (modularidade para montanha, cronograma, interfaces, riscos, anexos) e ZG-ONE-001 one-pager
- Janelas Olho recentradas nos vãos entre arcos (0,95 x 0,80 / 0,80 x 0,55) para os recortes não cruzarem o keder dos arcos; 00_BRIEFING/REVISOES.md criado
- regen.sh, README e especificação atualizados; regeneração completa

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXgeeezmv3d1TAAP83TAQH
</commit_message>
<xml_diff>
--- a/projects/zion-glamping-line/ZION_MATERIAIS_FFE_Linha.xlsx
+++ b/projects/zion-glamping-line/ZION_MATERIAIS_FFE_Linha.xlsx
@@ -15328,7 +15328,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11">
@@ -15348,7 +15348,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12">
@@ -15408,7 +15408,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15">
@@ -15428,7 +15428,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16">
@@ -15448,7 +15448,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17">
@@ -15468,7 +15468,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18">

</xml_diff>